<commit_message>
feat: harden comment quality validation
</commit_message>
<xml_diff>
--- a/references/样例-金样-40条.xlsx
+++ b/references/样例-金样-40条.xlsx
@@ -116,12 +116,12 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">我爸每天用百度查血压。</t>
+          <t xml:space="preserve">家里长辈常用百度查血压。</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">我妈也永远只会用百度…</t>
+          <t xml:space="preserve">家里长辈还是只会用百度…</t>
         </is>
       </c>
     </row>
@@ -138,7 +138,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">高血压吃什么、社保怎么交，这不就是我爸每天搜的吗？</t>
+          <t xml:space="preserve">高血压吃什么、社保怎么交，这不就是很多长辈每天搜的吗？</t>
         </is>
       </c>
     </row>
@@ -177,7 +177,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">我妈说八百遍让她换个AI她永远还是打开百度</t>
+          <t xml:space="preserve">提醒八百遍换个AI，家里长辈还是会打开百度</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -206,7 +206,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scaling Law早期证据也出自百度美研这段没几个人知道</t>
+          <t xml:space="preserve">一个公司走出这么多AI大佬，说明底子一直在，只是产品没接住，挺可惜的。</t>
         </is>
       </c>
     </row>
@@ -254,7 +254,7 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">一个公司走出这么多AI大佬，说明底子一直在，只是产品没接住，挺可惜的。</t>
+          <t xml:space="preserve">Scaling Law早期证据也出自百度美研这段没几个人知道</t>
         </is>
       </c>
     </row>
@@ -273,7 +273,7 @@
     <row r="15">
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">一线城市只有10.4%，难怪我身边一个用百度的都没有……</t>
+          <t xml:space="preserve">这个结论也不能一概而论</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -302,7 +302,7 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">我也是干这行的，看到这段手一抖。</t>
+          <t xml:space="preserve">做这行的人看到这段估计会手一抖。</t>
         </is>
       </c>
     </row>
@@ -333,7 +333,7 @@
     <row r="20">
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">杠精先别急着反驳</t>
+          <t xml:space="preserve">一线城市只有10.4%，难怪我身边一个用百度的都没有……</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">

</xml_diff>